<commit_message>
Add real class memories with overlapping photo pairs
</commit_message>
<xml_diff>
--- a/dm66-website/prebuilt/downloads/DM66D-memories-template.xlsx
+++ b/dm66-website/prebuilt/downloads/DM66D-memories-template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_dan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du_lieu_ky_niem" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vi_du_minh_hoa" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Huong_dan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Du_lieu_ky_niem" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vi_du_minh_hoa" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Du_lieu_ky_niem'!$A$1:$G$51</definedName>
@@ -594,7 +594,7 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Điền vào sheet Du_lieu_ky_niem. Mỗi dòng là một kỷ niệm và một ảnh. Sheet dữ liệu đang để trống để bạn nhập nội dung thật của lớp.</t>
+          <t>Điền vào sheet Du_lieu_ky_niem. Mỗi dòng là một sự kiện với hai ảnh. Sheet dữ liệu đang để trống để bạn nhập nội dung thật của lớp.</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>1. File Excel này sau khi điền.
-2. File anh-ky-niem.zip chứa các ảnh gốc. Tên từng ảnh trong ZIP phải khớp chính xác với cột image, kể cả phần mở rộng.</t>
+2. File anh-ky-niem.zip chứa ảnh gốc JPEG. Mỗi sự kiện có hai tên ảnh trong cột image, mỗi tên một dòng; tên phải khớp file trong ZIP.</t>
         </is>
       </c>
     </row>
@@ -624,9 +624,9 @@
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>id: mã duy nhất, không trùng; nên dùng ky-niem-01, ky-niem-02…
-title: tên kỷ niệm.
-image: tên file ảnh, ví dụ ky-niem-01.jpg.
-description: lời mô tả 2–4 câu, dựa trên thông tin thật do lớp cung cấp.</t>
+title: tên sự kiện đầy đủ.
+image: hai tên file JPEG, mỗi tên một dòng bằng Alt+Enter.
+description: mô tả đầy đủ dựa trên nội dung thật của lớp; giữ nguyên cách viết.</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
     <row r="20" ht="58" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Ưu tiên ảnh ngang 16:9 hoặc 3:2, đủ nét; định dạng .jpg, .jpeg, .png hoặc .webp. Một dòng chỉ ghi một tên ảnh. Có thể dùng lại một ảnh cho nhiều dòng nếu cần. Nên dùng tên file đơn giản, không dấu, không khoảng trắng.</t>
+          <t>Mỗi sự kiện dùng hai ảnh .jpg hoặc .jpeg. Trong cột image, ghi mỗi tên ảnh trên một dòng bằng Alt+Enter. Bố cục giữ tỷ lệ ảnh gốc; có thể dùng ảnh ngang, vuông hoặc dọc. Nên dùng tên file đơn giản, không dấu.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <row r="23" ht="58" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Không chèn ảnh trực tiếp vào ô Excel. Không ghi đường dẫn C:\…, /Users/…, /workspace/… hoặc liên kết riêng trên máy. Cột image chỉ cần tên file có phần mở rộng; đặt các ảnh trực tiếp trong ZIP để đối chiếu dễ dàng.</t>
+          <t>Không chèn ảnh trực tiếp vào ô Excel. Không ghi đường dẫn trên máy hoặc liên kết riêng. Cột image chỉ ghi hai tên file có phần mở rộng, mỗi tên một dòng; các ảnh nằm trong ZIP gửi kèm.</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
     <row r="29" ht="58" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Mỗi dòng đã điền đủ bốn cột có dấu *. Không có id trùng. Tên ảnh khớp với file trong ZIP. Tiếng Việt có dấu đúng. Ảnh và nội dung đã được lớp đồng ý chia sẻ công khai.</t>
+          <t>Tên sự kiện được viết đầy đủ, id không trùng. Mỗi sự kiện có hai tên ảnh trong cột image, khớp với file JPEG trong ZIP. Tiếng Việt có dấu đúng. Ảnh và nội dung đã được lớp đồng ý chia sẻ công khai.</t>
         </is>
       </c>
     </row>

</xml_diff>